<commit_message>
[ENH] SF image generation from psychopy, updated GUI and minor bug solving
</commit_message>
<xml_diff>
--- a/src/instructions/BL4_instructions.xlsx
+++ b/src/instructions/BL4_instructions.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27928"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28730"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\akoun\Desktop\Biocruces\siburmuin\src\begiBrainDemo\instructions\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\akoun\Desktop\Biocruces\begibraintool\src\instructions\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A5CA77C1-7C22-4FF6-B433-32270F1A253E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9C65A07D-4509-4D5D-851D-AFA32850A8E5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -96,7 +96,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="8">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10" uniqueCount="10">
   <si>
     <t>title</t>
   </si>
@@ -116,10 +116,16 @@
     <t>instruction_5</t>
   </si>
   <si>
-    <t>Debes usar las flechas del teclado (derecha/izquierda) para responder a la siguiente pregunta: ¿Qué orientación tiene el parche? Solo tienes 2 segundos para ver el estímulo.</t>
-  </si>
-  <si>
-    <t>BLOQUE 4: FLICKER</t>
+    <t>BLOQUE 5: ESTÍMULOS SEMÁNTICOS - FRECUENCIA ESPACIAL</t>
+  </si>
+  <si>
+    <t>A continuación vas a ver una série de imágenes. Para cada imagen que se muestre debes responder si se trata de un ser vivo o un objeto inerte.</t>
+  </si>
+  <si>
+    <t>Las imágenes no se van a ver al completo, hemos modificado unos parámetros para hacerlo un poco más dificil.</t>
+  </si>
+  <si>
+    <t>Pulsa el botón central para empezar la prueba.</t>
   </si>
 </sst>
 </file>
@@ -550,10 +556,16 @@
     </row>
     <row r="2" spans="1:6" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A2" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="B2" t="s">
         <v>7</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>6</v>
+        <v>8</v>
+      </c>
+      <c r="D2" t="s">
+        <v>9</v>
       </c>
     </row>
   </sheetData>
@@ -569,21 +581,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100B9F5CAB0486A994CA2C3B13E059EF2AE" ma:contentTypeVersion="0" ma:contentTypeDescription="Een nieuw document maken." ma:contentTypeScope="" ma:versionID="8645ec4a60d0c8c7009d2d6675847a91">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="636d7205651659ec4fcda0bcbde9384b">
     <xsd:element name="properties">
@@ -697,30 +694,22 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B3725960-8A89-4E70-9C40-340E0EDB6403}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{3744155D-8FAB-4E67-B5E0-C7FDBFB3715D}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{EFF1C174-6AC6-4774-A736-3226A12360E4}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -734,4 +723,27 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{3744155D-8FAB-4E67-B5E0-C7FDBFB3715D}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B3725960-8A89-4E70-9C40-340E0EDB6403}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
[ENH] Added module 5 + bug solving during feedback and noise time
</commit_message>
<xml_diff>
--- a/src/instructions/BL4_instructions.xlsx
+++ b/src/instructions/BL4_instructions.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\akoun\Desktop\Biocruces\begibraintool\src\instructions\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9C65A07D-4509-4D5D-851D-AFA32850A8E5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C98363FB-26BF-4B9D-9E92-07EB22390C4A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="43080" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -116,9 +116,6 @@
     <t>instruction_5</t>
   </si>
   <si>
-    <t>BLOQUE 5: ESTÍMULOS SEMÁNTICOS - FRECUENCIA ESPACIAL</t>
-  </si>
-  <si>
     <t>A continuación vas a ver una série de imágenes. Para cada imagen que se muestre debes responder si se trata de un ser vivo o un objeto inerte.</t>
   </si>
   <si>
@@ -126,6 +123,9 @@
   </si>
   <si>
     <t>Pulsa el botón central para empezar la prueba.</t>
+  </si>
+  <si>
+    <t>BLOQUE 4: ESTÍMULOS SEMÁNTICOS - FRECUENCIA ESPACIAL</t>
   </si>
 </sst>
 </file>
@@ -556,16 +556,16 @@
     </row>
     <row r="2" spans="1:6" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A2" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="B2" t="s">
         <v>6</v>
       </c>
-      <c r="B2" t="s">
+      <c r="C2" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="C2" s="3" t="s">
+      <c r="D2" t="s">
         <v>8</v>
-      </c>
-      <c r="D2" t="s">
-        <v>9</v>
       </c>
     </row>
   </sheetData>
@@ -581,6 +581,21 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100B9F5CAB0486A994CA2C3B13E059EF2AE" ma:contentTypeVersion="0" ma:contentTypeDescription="Een nieuw document maken." ma:contentTypeScope="" ma:versionID="8645ec4a60d0c8c7009d2d6675847a91">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="636d7205651659ec4fcda0bcbde9384b">
     <xsd:element name="properties">
@@ -694,22 +709,30 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
-</file>
-
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B3725960-8A89-4E70-9C40-340E0EDB6403}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{3744155D-8FAB-4E67-B5E0-C7FDBFB3715D}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{EFF1C174-6AC6-4774-A736-3226A12360E4}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -723,27 +746,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{3744155D-8FAB-4E67-B5E0-C7FDBFB3715D}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B3725960-8A89-4E70-9C40-340E0EDB6403}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>